<commit_message>
Frissített forgalmi munkafüzet (javítási típusok lappal)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Votz75dLaDY1wx33JY26GU
</commit_message>
<xml_diff>
--- a/dokumentumok/forgalmi_munkafuzet.xlsx
+++ b/dokumentumok/forgalmi_munkafuzet.xlsx
@@ -5,6 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="120" yWindow="75" windowWidth="21075" windowHeight="8265" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="105" windowWidth="27795" windowHeight="12600" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Adatok" sheetId="1" r:id="rId1"/>
@@ -15,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>Hónap</t>
   </si>
@@ -120,13 +121,76 @@
   </si>
   <si>
     <t>Legkisebb kiadási kategória</t>
+  </si>
+  <si>
+    <t>Javítás típusa</t>
+  </si>
+  <si>
+    <t>Javítások száma (db)</t>
+  </si>
+  <si>
+    <t>Kezdő ár (Ft)</t>
+  </si>
+  <si>
+    <t>Kijelzőcsere</t>
+  </si>
+  <si>
+    <t>Akkumulátorcsere</t>
+  </si>
+  <si>
+    <t>Töltőcsatlakozó csere</t>
+  </si>
+  <si>
+    <t>Hátlapcsere</t>
+  </si>
+  <si>
+    <t>Szoftveres hibaelhárítás</t>
+  </si>
+  <si>
+    <t>Vízkár-kezelés</t>
+  </si>
+  <si>
+    <t>Kijelzőcserék százaléka</t>
+  </si>
+  <si>
+    <t>Akkumulátorcserék százaléka</t>
+  </si>
+  <si>
+    <t>Töltőcsatlakozó cserék százaléka</t>
+  </si>
+  <si>
+    <t>Hátlapcserék százaléka</t>
+  </si>
+  <si>
+    <t>Szoftveres hibaelhárítások százaléka</t>
+  </si>
+  <si>
+    <t>Vízkár-kezelések százaléka</t>
+  </si>
+  <si>
+    <t>Kijelzőcserék becsült bevétele</t>
+  </si>
+  <si>
+    <t>Akkumulátorcserék becsült bevétele</t>
+  </si>
+  <si>
+    <t>Töltőcsatlakozó cserék becsült bevétele</t>
+  </si>
+  <si>
+    <t>Hátlapcserék becsült bevétele</t>
+  </si>
+  <si>
+    <t>Szoftveres hibaelhárítások becsült bevétele</t>
+  </si>
+  <si>
+    <t>Vízkár-kezelések becsült bevétele</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,6 +211,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -193,10 +270,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -210,20 +288,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF1F3864"/>
       <color rgb="FF92AEE2"/>
       <color rgb="FF7EA2DA"/>
       <color rgb="FF6694D0"/>
+      <color rgb="FF2E79BA"/>
       <color rgb="FF27578E"/>
-      <color rgb="FF2E79BA"/>
+      <color rgb="FF1F3864"/>
       <color rgb="FFC3C3C3"/>
     </mruColors>
   </colors>
@@ -538,11 +621,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="155842048"/>
-        <c:axId val="150175744"/>
+        <c:axId val="211762688"/>
+        <c:axId val="167935296"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="155842048"/>
+        <c:axId val="211762688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -551,7 +634,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="150175744"/>
+        <c:crossAx val="167935296"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -559,7 +642,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="150175744"/>
+        <c:axId val="167935296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -570,7 +653,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="155842048"/>
+        <c:crossAx val="211762688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -656,7 +739,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Adatok!$G$1</c:f>
+              <c:f>Adatok!$J$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -834,7 +917,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Adatok!$F$2:$G$7</c:f>
+              <c:f>Adatok!$I$2:$J$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="6"/>
                 <c:lvl>
@@ -882,7 +965,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Adatok!$G$2:$G$7</c:f>
+              <c:f>Adatok!$J$2:$J$7</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="6"/>
@@ -945,6 +1028,366 @@
     <c:pageSetup/>
   </c:printSettings>
   <c:userShapes r:id="rId1"/>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="5.9391951006124231E-2"/>
+          <c:y val="0.14803258967629046"/>
+          <c:w val="0.53010826771653541"/>
+          <c:h val="0.68969123651210262"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Kijelzőcsere</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3864"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$16</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.34</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Akkumulátorcsere</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="27578E"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$18</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.26</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Töltőcsatlakozó csere</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E79BA"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$20</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Hátlapcsere</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="6694D0"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$22</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Szoftveres hibaelhárítás</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7EA2DA"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$24</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.09</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Adatok!$E$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Vízkár-kezelés</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="92AEE2"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Összesítés!$C$26</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="151376384"/>
+        <c:axId val="151132352"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="151376384"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="151132352"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="151132352"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="151376384"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.64750034556784553"/>
+          <c:y val="0.12558636363636366"/>
+          <c:w val="0.3286155094610364"/>
+          <c:h val="0.74613080808080801"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
@@ -991,7 +1434,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>47624</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>107156</xdr:rowOff>
+      <xdr:rowOff>116672</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1005,6 +1448,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>53578</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>21433</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>40246</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>96433</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1355,17 +1828,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="2" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="1" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="10" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1376,15 +1849,24 @@
         <v>2</v>
       </c>
       <c r="D1" s="2"/>
+      <c r="E1" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="F1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="2"/>
+      <c r="I1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
@@ -1395,15 +1877,24 @@
         <v>1059000</v>
       </c>
       <c r="D2" s="3"/>
-      <c r="F2" s="6" t="s">
+      <c r="E2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="7">
+        <v>476</v>
+      </c>
+      <c r="G2" s="7">
+        <v>18900</v>
+      </c>
+      <c r="H2" s="5"/>
+      <c r="I2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="7">
+      <c r="J2" s="7">
         <v>5600000</v>
       </c>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
@@ -1414,15 +1905,24 @@
         <v>1077000</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="F3" s="9" t="s">
+      <c r="E3" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="10">
+        <v>364</v>
+      </c>
+      <c r="G3" s="10">
+        <v>9900</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="10">
+      <c r="J3" s="10">
         <v>4800000</v>
       </c>
-      <c r="H3" s="5"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -1433,15 +1933,24 @@
         <v>1132000</v>
       </c>
       <c r="D4" s="3"/>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="7">
+        <v>196</v>
+      </c>
+      <c r="G4" s="7">
+        <v>8900</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="7">
+      <c r="J4" s="7">
         <v>1920000</v>
       </c>
-      <c r="H4" s="5"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
@@ -1452,15 +1961,24 @@
         <v>1110000</v>
       </c>
       <c r="D5" s="3"/>
-      <c r="F5" s="9" t="s">
+      <c r="E5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="10">
+        <v>140</v>
+      </c>
+      <c r="G5" s="10">
+        <v>11900</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="10">
+      <c r="J5" s="10">
         <v>540000</v>
       </c>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -1471,15 +1989,24 @@
         <v>1159000</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="F6" s="6" t="s">
+      <c r="E6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="7">
+        <v>126</v>
+      </c>
+      <c r="G6" s="7">
+        <v>5900</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="7">
+      <c r="J6" s="7">
         <v>480000</v>
       </c>
-      <c r="H6" s="5"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>8</v>
       </c>
@@ -1490,15 +2017,24 @@
         <v>1150000</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="F7" s="9" t="s">
+      <c r="E7" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="10">
+        <v>98</v>
+      </c>
+      <c r="G7" s="10">
+        <v>12900</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="10">
+      <c r="J7" s="10">
         <v>660000</v>
       </c>
-      <c r="H7" s="5"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -1513,7 +2049,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
@@ -1525,7 +2061,7 @@
       </c>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
@@ -1536,8 +2072,10 @@
         <v>1223000</v>
       </c>
       <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="11"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
@@ -1548,8 +2086,9 @@
         <v>1214000</v>
       </c>
       <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
@@ -1560,8 +2099,10 @@
         <v>1256000</v>
       </c>
       <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F12" s="14"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>14</v>
       </c>
@@ -1572,12 +2113,29 @@
         <v>1323000</v>
       </c>
       <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F13" s="14"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
+      <c r="F14" s="14"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F15" s="14"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H18" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1587,7 +2145,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:D16"/>
+  <dimension ref="B2:D27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1706,7 +2264,7 @@
         <v>33</v>
       </c>
       <c r="C13" t="str">
-        <f>INDEX(Adatok!F2:G7,MATCH(MAX(Adatok!G2:G7),Adatok!G2:G7,0),1)</f>
+        <f>INDEX(Adatok!I2:J7,MATCH(MAX(Adatok!J2:J7),Adatok!J2:J7,0),1)</f>
         <v>Alkatrészek</v>
       </c>
     </row>
@@ -1715,12 +2273,118 @@
         <v>34</v>
       </c>
       <c r="C14" s="1" t="str">
-        <f>INDEX(Adatok!F2:G7,MATCH(MIN(Adatok!G2:G7),Adatok!G2:G7,0),1)</f>
+        <f>INDEX(Adatok!I2:J7,MATCH(MIN(Adatok!J2:J7),Adatok!J2:J7,0),1)</f>
         <v>Marketing</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="12">
+        <f>Adatok!F2/SUM(Adatok!$F$2:$F$7)</f>
+        <v>0.34</v>
+      </c>
       <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1">
+        <f>Adatok!F2*Adatok!G2</f>
+        <v>8996400</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="12">
+        <f>Adatok!F3/SUM(Adatok!$F$2:$F$7)</f>
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="1">
+        <f>Adatok!F3*Adatok!G3</f>
+        <v>3603600</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="12">
+        <f>Adatok!F4/SUM(Adatok!$F$2:$F$7)</f>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="1">
+        <f>Adatok!F4*Adatok!G4</f>
+        <v>1744400</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="12">
+        <f>Adatok!F5/SUM(Adatok!$F$2:$F$7)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="1">
+        <f>Adatok!F5*Adatok!G5</f>
+        <v>1666000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="12">
+        <f>Adatok!F6/SUM(Adatok!$F$2:$F$7)</f>
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="1">
+        <f>Adatok!F6*Adatok!G6</f>
+        <v>743400</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="12">
+        <f>Adatok!F7/SUM(Adatok!$F$2:$F$7)</f>
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="1">
+        <f>Adatok!F7*Adatok!G7</f>
+        <v>1264200</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>